<commit_message>
feat: เปลี่ยน 3CX→Phonebook, Website→Software, ลบ Intranet (แนวทาง B)
- DB: ALTER TABLE Employee RENAME phone3cx→phonebook, website→software, DROP intranet/intranetDate
- prisma/schema.prisma: อัปเดต field names ให้ตรงกับ DB ใหม่
- employees.ts: HEADER_MAP, filters, POST/PATCH ใช้ field ใหม่ทั้งหมด
- dashboard.ts: select + isItCleared ใช้ field ใหม่
- reports.ts: isItCleared, column defs, headers, values (19 cols แทน 21)
- AllRecordsPage: interface, HEADERS, state vars, fetchData params, table cells, modal
- AddRecordPage/EditRecordPage: fields array, IT_KEYS, IT_DATE_KEYS, IT_TO_DATE
- Excel template: ปรับหัวคอลัมน์ Website→Software, 3CX→Phonebook, ลบ Intranet

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -398,17 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="32.83203125" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
feat: อัปเดต Excel template ใหม่รองรับ DataSource columns
เพิ่มคอลัมน์ ข้อมูลต้นทาง/เดือน/ปี/วันที่ได้รับข้อมูล
และ script สำหรับ regenerate template

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -1,58 +1,185 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="employees" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Template" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="42">
+  <si>
+    <t>ข้อมูลต้นทาง</t>
+  </si>
+  <si>
+    <t>เดือน</t>
+  </si>
+  <si>
+    <t>ปี</t>
+  </si>
+  <si>
+    <t>วันที่ได้รับข้อมูล</t>
+  </si>
+  <si>
+    <t>รหัสประจำตัว</t>
+  </si>
+  <si>
+    <t>ชื่อ-สกุล</t>
+  </si>
+  <si>
+    <t>Name-Eng</t>
+  </si>
+  <si>
+    <t>ตำแหน่ง</t>
+  </si>
+  <si>
+    <t>ประเภท</t>
+  </si>
+  <si>
+    <t>ฝ่าย/กลุ่ม/งาน</t>
+  </si>
+  <si>
+    <t>หน่วยงาน</t>
+  </si>
+  <si>
+    <t>วันที่พ้นสภาพ</t>
+  </si>
+  <si>
+    <t>วันเริ่มงาน</t>
+  </si>
+  <si>
+    <t>FMIS</t>
+  </si>
+  <si>
+    <t>eMeeting</t>
+  </si>
+  <si>
+    <t>Software</t>
+  </si>
+  <si>
+    <t>Phonebook</t>
+  </si>
+  <si>
+    <t>1=สบค., 2=ศล.</t>
+  </si>
+  <si>
+    <t>1-12</t>
+  </si>
+  <si>
+    <t>พ.ศ. เช่น 2567</t>
+  </si>
+  <si>
+    <t>วัน/เดือน/ปี พ.ศ.</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ</t>
+  </si>
+  <si>
+    <t>15/6/2568</t>
+  </si>
+  <si>
+    <t>EMP001</t>
+  </si>
+  <si>
+    <t>สมชาย ใจดี</t>
+  </si>
+  <si>
+    <t>Somchai Jaidee</t>
+  </si>
+  <si>
+    <t>นักวิชาการคอมพิวเตอร์</t>
+  </si>
+  <si>
+    <t>ข้าราชการ</t>
+  </si>
+  <si>
+    <t>ฝ่ายเทคโนโลยีสารสนเทศ</t>
+  </si>
+  <si>
+    <t>สำนักงานบริหารทรัพยากรบุคคล</t>
+  </si>
+  <si>
+    <t>30/6/2568</t>
+  </si>
+  <si>
+    <t>ดำเนินการแล้ว</t>
+  </si>
+  <si>
+    <t>ยังไม่ดำเนินการ</t>
+  </si>
+  <si>
+    <t>EMP002</t>
+  </si>
+  <si>
+    <t>สมหญิง รักงาน</t>
+  </si>
+  <si>
+    <t>Somying Rakngam</t>
+  </si>
+  <si>
+    <t>เจ้าหน้าที่บริหารงานทั่วไป</t>
+  </si>
+  <si>
+    <t>ลูกจ้างประจำ</t>
+  </si>
+  <si>
+    <t>ฝ่ายบริหาร</t>
+  </si>
+  <si>
+    <t>ศูนย์บริการโลหิตแห่งชาติ</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D4ED8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +187,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,70 +545,238 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="17" width="12" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ชื่อไฟล์</v>
-      </c>
-      <c r="B1" t="str">
-        <v>รหัสประจำตัว</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ชื่อ-สกุล</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Name-Eng</v>
-      </c>
-      <c r="E1" t="str">
-        <v>ตำแหน่ง</v>
-      </c>
-      <c r="F1" t="str">
-        <v>ประเภท</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ฝ่าย/กลุ่ม/งาน</v>
-      </c>
-      <c r="H1" t="str">
-        <v>หน่วยงาน</v>
-      </c>
-      <c r="I1" t="str">
-        <v>วันที่พ้นสภาพ</v>
+    <row r="1" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>พ้นสภาพ_รอบปี_2595.xlsx</v>
-      </c>
-      <c r="B2" t="str">
-        <v>5690267</v>
-      </c>
-      <c r="C2" t="str">
-        <v>นาย พรเพชร นาคำภา</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Mr. Pornpetch Nakumpa</v>
-      </c>
-      <c r="E2" t="str">
-        <v>เจ้าหน้าที่พัฒนาระบบ</v>
-      </c>
-      <c r="F2" t="str">
-        <v>เจ้าหน้าที่</v>
-      </c>
-      <c r="G2" t="str">
-        <v>ฝ่ายบริการและสนับสนุนซอฟต์แวร์</v>
-      </c>
-      <c r="H2" t="str">
-        <v>สำนักงานเทคโนโลยีสารสนเทศและดิจิทัล</v>
-      </c>
-      <c r="I2" t="str">
-        <v>1/2/2595</v>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2568</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2568</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: remove 'required' text and example rows from import template
Note rows with 'required' in employeeId/nameTh columns were being
imported as real records. Clear those cells and remove example rows.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -61,58 +61,7 @@
     <t>วัน/เดือน/ปี พ.ศ.</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
     <t/>
-  </si>
-  <si>
-    <t>15/6/2568</t>
-  </si>
-  <si>
-    <t>EMP001</t>
-  </si>
-  <si>
-    <t>สมชาย ใจดี</t>
-  </si>
-  <si>
-    <t>Somchai Jaidee</t>
-  </si>
-  <si>
-    <t>นักวิชาการคอมพิวเตอร์</t>
-  </si>
-  <si>
-    <t>ข้าราชการ</t>
-  </si>
-  <si>
-    <t>ฝ่ายเทคโนโลยีสารสนเทศ</t>
-  </si>
-  <si>
-    <t>สำนักงานบริหารทรัพยากรบุคคล</t>
-  </si>
-  <si>
-    <t>30/6/2568</t>
-  </si>
-  <si>
-    <t>EMP002</t>
-  </si>
-  <si>
-    <t>สมหญิง รักงาน</t>
-  </si>
-  <si>
-    <t>Somying Rakngam</t>
-  </si>
-  <si>
-    <t>เจ้าหน้าที่บริหารงานทั่วไป</t>
-  </si>
-  <si>
-    <t>ลูกจ้างประจำ</t>
-  </si>
-  <si>
-    <t>ฝ่ายบริหาร</t>
-  </si>
-  <si>
-    <t>ศูนย์บริการโลหิตแห่งชาติ</t>
   </si>
 </sst>
 </file>
@@ -174,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -182,7 +131,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -522,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -594,98 +542,22 @@
         <v>16</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3">
-        <v>6</v>
-      </c>
-      <c r="C3" s="3">
-        <v>2568</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3">
-        <v>6</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2568</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add อีเมล column to Excel import template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -49,6 +49,9 @@
     <t>วันที่พ้นสภาพ</t>
   </si>
   <si>
+    <t>อีเมล</t>
+  </si>
+  <si>
     <t>1=สบค., 2=ศล.</t>
   </si>
   <si>
@@ -62,6 +65,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>example@email.com</t>
   </si>
 </sst>
 </file>
@@ -470,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -482,9 +488,10 @@
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -521,47 +528,53 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>15</v>
+      <c r="M2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add sample data row to Excel import template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -52,22 +52,31 @@
     <t>อีเมล</t>
   </si>
   <si>
-    <t>1=สบค., 2=ศล.</t>
-  </si>
-  <si>
-    <t>1-12</t>
-  </si>
-  <si>
-    <t>พ.ศ. เช่น 2567</t>
-  </si>
-  <si>
-    <t>วัน/เดือน/ปี พ.ศ.</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>example@email.com</t>
+    <t>31/3/2599</t>
+  </si>
+  <si>
+    <t>5690267</t>
+  </si>
+  <si>
+    <t>พรเพชร นาคำภา</t>
+  </si>
+  <si>
+    <t>Pornpetch Nakumpa</t>
+  </si>
+  <si>
+    <t>เจ้าหน้าที่พัฒนาระบบ</t>
+  </si>
+  <si>
+    <t>เจ้าหน้าที่</t>
+  </si>
+  <si>
+    <t>ฝ่ายบริการและสนับสนุนซอฟต์แวร์</t>
+  </si>
+  <si>
+    <t>สำนักงานเทคโนโลยีสารสนเทศและดิจิทัล</t>
+  </si>
+  <si>
+    <t>pornpetch.n@redcross.or.th</t>
   </si>
 </sst>
 </file>
@@ -87,9 +96,8 @@
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
-      <i/>
-      <color rgb="FF64748B"/>
-      <sz val="9"/>
+      <sz val="12"/>
+      <name val="TH SarabunPSK"/>
     </font>
   </fonts>
   <fills count="4">
@@ -106,11 +114,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -125,6 +133,17 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -134,8 +153,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -532,45 +551,45 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2599</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: restore hint row in import template, keep sample data as row 3
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/employee_import_template.xlsx
+++ b/public/employee_import_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -50,6 +50,21 @@
   </si>
   <si>
     <t>อีเมล</t>
+  </si>
+  <si>
+    <t>1=สบค., 2=ศล.</t>
+  </si>
+  <si>
+    <t>1-12</t>
+  </si>
+  <si>
+    <t>พ.ศ. เช่น 2567</t>
+  </si>
+  <si>
+    <t>วัน/เดือน/ปี พ.ศ.</t>
+  </si>
+  <si>
+    <t>example@email.com</t>
   </si>
   <si>
     <t>31/3/2599</t>
@@ -83,7 +98,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -96,11 +111,17 @@
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
+      <i/>
+      <color rgb="FF6B7280"/>
+      <sz val="11"/>
+      <name val="TH SarabunPSK"/>
+    </font>
+    <font>
       <sz val="12"/>
       <name val="TH SarabunPSK"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -114,11 +135,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -136,6 +162,17 @@
     <border>
       <left/>
       <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color rgb="FFD1D5DB"/>
       </right>
       <top/>
@@ -148,12 +185,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -495,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -551,45 +591,72 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" ht="18" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B3" s="3">
         <v>3</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C3" s="3">
         <v>2599</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>21</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>